<commit_message>
url is getting from config
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Results.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Results.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="294">
   <si>
     <t>Test Data</t>
   </si>
@@ -861,13 +861,109 @@
   <si>
     <t>2026-03-03 14:15:47</t>
   </si>
+  <si>
+    <t>69a6a94ec46935d1717e1505</t>
+  </si>
+  <si>
+    <t>2026-03-03 14:57:19</t>
+  </si>
+  <si>
+    <t>69a6aa08c46935d1717e1c57</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:00:27</t>
+  </si>
+  <si>
+    <t>69a6aaa3c46935d1717e1fff</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:03:01</t>
+  </si>
+  <si>
+    <t>69a6aaedc46935d1717e23ba</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:04:13</t>
+  </si>
+  <si>
+    <t>69a6ab63c46935d1717e2764</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:06:13</t>
+  </si>
+  <si>
+    <t>69a6aba8c46935d1717e2b06</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:07:22</t>
+  </si>
+  <si>
+    <t>123 Main Street</t>
+  </si>
+  <si>
+    <t>69a6ac6fc46935d1717e3261</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:10:44</t>
+  </si>
+  <si>
+    <t>69a6ad4ac46935d1717e3637</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:14:23</t>
+  </si>
+  <si>
+    <t>560001</t>
+  </si>
+  <si>
+    <t>69a6ad9bc46935d1717e39f3</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:15:41</t>
+  </si>
+  <si>
+    <t>10001</t>
+  </si>
+  <si>
+    <t>69a6ade7c46935d1717e40e6</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:16:58</t>
+  </si>
+  <si>
+    <t>90210</t>
+  </si>
+  <si>
+    <t>69a6ae3fc46935d1717e47d6</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:18:25</t>
+  </si>
+  <si>
+    <t>SW1A 1AA</t>
+  </si>
+  <si>
+    <t>69a6ae98c46935d1717e4b94</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:19:53</t>
+  </si>
+  <si>
+    <t>H0H 0H0</t>
+  </si>
+  <si>
+    <t>69a6aeebc46935d1717e52d3</t>
+  </si>
+  <si>
+    <t>2026-03-03 15:21:16</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="332" x14ac:knownFonts="1">
+  <fonts count="371" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -897,6 +993,227 @@
       <sz val="11"/>
       <color indexed="9"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -2792,7 +3109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="332">
+  <cellXfs count="371">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3785,6 +4102,123 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="331" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="332" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="333" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="334" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="335" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="336" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="337" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="338" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="339" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="340" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="341" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="342" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="343" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="344" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="345" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="346" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="347" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="348" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="349" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="350" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="351" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="352" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="353" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="354" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="355" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="356" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="357" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="358" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="359" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="360" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="361" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="362" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="363" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="364" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="365" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="366" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="367" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="368" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="369" fillId="4" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="370" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4130,7 +4564,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="22.7265625"/>
@@ -7001,6 +7435,344 @@
       </c>
       <c r="H112" t="s" s="0">
         <v>261</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B113" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C113" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D113" s="333" t="s">
+        <v>26</v>
+      </c>
+      <c r="E113" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="F113" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G113" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H113" t="s" s="0">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B114" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C114" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D114" s="336" t="s">
+        <v>26</v>
+      </c>
+      <c r="E114" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="F114" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G114" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H114" t="s" s="0">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B115" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C115" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D115" s="339" t="s">
+        <v>26</v>
+      </c>
+      <c r="E115" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="F115" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G115" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H115" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D116" s="342" t="s">
+        <v>26</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>268</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G116" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H116" t="s" s="0">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D117" s="345" t="s">
+        <v>26</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>270</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G117" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H117" t="s" s="0">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B118" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C118" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D118" s="348" t="s">
+        <v>26</v>
+      </c>
+      <c r="E118" t="s" s="0">
+        <v>272</v>
+      </c>
+      <c r="F118" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G118" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H118" t="s" s="0">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s" s="0">
+        <v>274</v>
+      </c>
+      <c r="B119" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C119" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D119" s="351" t="s">
+        <v>208</v>
+      </c>
+      <c r="E119" t="s" s="0">
+        <v>275</v>
+      </c>
+      <c r="F119" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G119" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H119" t="s" s="0">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B120" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C120" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D120" s="354" t="s">
+        <v>208</v>
+      </c>
+      <c r="E120" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="F120" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G120" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H120" t="s" s="0">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="B121" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C121" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D121" s="357" t="s">
+        <v>208</v>
+      </c>
+      <c r="E121" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="F121" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G121" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H121" t="s" s="0">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B122" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C122" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D122" s="360" t="s">
+        <v>208</v>
+      </c>
+      <c r="E122" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="F122" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G122" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H122" t="s" s="0">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="B123" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C123" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D123" s="363" t="s">
+        <v>208</v>
+      </c>
+      <c r="E123" t="s" s="0">
+        <v>286</v>
+      </c>
+      <c r="F123" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G123" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H123" t="s" s="0">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s" s="0">
+        <v>288</v>
+      </c>
+      <c r="B124" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C124" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D124" s="366" t="s">
+        <v>208</v>
+      </c>
+      <c r="E124" t="s" s="0">
+        <v>289</v>
+      </c>
+      <c r="F124" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G124" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H124" t="s" s="0">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s" s="0">
+        <v>291</v>
+      </c>
+      <c r="B125" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C125" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D125" s="369" t="s">
+        <v>208</v>
+      </c>
+      <c r="E125" t="s" s="0">
+        <v>292</v>
+      </c>
+      <c r="F125" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="G125" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H125" t="s" s="0">
+        <v>293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rin for payaza cards
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Results.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Results.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1821" uniqueCount="529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1845" uniqueCount="536">
   <si>
     <t>Test Data</t>
   </si>
@@ -1816,13 +1816,34 @@
   <si>
     <t>2026-03-20 11:00:41</t>
   </si>
+  <si>
+    <t>FAIL → Exception occurred during payment flow: java.lang.RuntimeException: ✗ selectAuthResult dropdown NOT found in any iframe!</t>
+  </si>
+  <si>
+    <t>69bcdc2b31f5cace0479feca</t>
+  </si>
+  <si>
+    <t>2026-03-20 11:05:16</t>
+  </si>
+  <si>
+    <t>69bcde1731f5cace047a0ed7</t>
+  </si>
+  <si>
+    <t>2026-03-20 11:12:32</t>
+  </si>
+  <si>
+    <t>69bcdebf31f5cace047a12b1</t>
+  </si>
+  <si>
+    <t>2026-03-20 11:15:22</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="267" x14ac:knownFonts="1">
+  <fonts count="276" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3135,6 +3156,57 @@
       <sz val="11"/>
       <color indexed="9"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -3449,7 +3521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="267">
+  <cellXfs count="276">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4247,6 +4319,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="266" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="267" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="268" fillId="3" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="269" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="270" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="271" fillId="3" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="272" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="273" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="274" fillId="3" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="275" fillId="2" borderId="0" xfId="0" applyFill="true" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4592,7 +4691,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H230"/>
+  <dimension ref="A1:H233"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="22.7265625"/>
@@ -10430,6 +10529,84 @@
       </c>
       <c r="H230" t="s" s="0">
         <v>528</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B231" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C231" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D231" s="269" t="s">
+        <v>529</v>
+      </c>
+      <c r="E231" t="s" s="0">
+        <v>530</v>
+      </c>
+      <c r="F231" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="G231" t="s" s="0">
+        <v>527</v>
+      </c>
+      <c r="H231" t="s" s="0">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B232" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C232" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D232" s="271" t="s">
+        <v>208</v>
+      </c>
+      <c r="E232" t="s" s="0">
+        <v>532</v>
+      </c>
+      <c r="F232" t="s" s="0">
+        <v>527</v>
+      </c>
+      <c r="G232" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H232" t="s" s="0">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B233" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C233" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D233" s="274" t="s">
+        <v>26</v>
+      </c>
+      <c r="E233" t="s" s="0">
+        <v>534</v>
+      </c>
+      <c r="F233" t="s" s="0">
+        <v>527</v>
+      </c>
+      <c r="G233" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="H233" t="s" s="0">
+        <v>535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>